<commit_message>
Truncate percentage displays instead of rounding, fix profit-row decimal display
Percentage cells (margin/checksum rows, dividend yield) now truncate to
1 decimal via TRUNC/math.trunc before display, since relying on the
cell's display format alone rounds half-up. Also fixed profit rows
(9-12) which had an integer-only number format despite storing
2-decimal values, silently rounding e.g. 137.61 to 138 on screen.
</commit_message>
<xml_diff>
--- a/templates/execution_table_template.xlsx
+++ b/templates/execution_table_template.xlsx
@@ -15,7 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="0.00_);[Red]\(0.00\)"/>
     <numFmt numFmtId="165" formatCode="0;[Red]\(0\);\-"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -23,6 +23,7 @@
     <numFmt numFmtId="168" formatCode="#,##0_);[Red]▲#,##0"/>
     <numFmt numFmtId="169" formatCode="0;[Red]▲0;-"/>
     <numFmt numFmtId="170" formatCode="0.0_);[Red]▲0.0_)"/>
+    <numFmt numFmtId="171" formatCode="0.00;[Red]▲0.00;-"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -689,7 +690,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="192">
+  <cellXfs count="201">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1229,6 +1230,33 @@
     </xf>
     <xf numFmtId="170" fontId="5" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1857,43 +1885,43 @@
           <t>第1四半期</t>
         </is>
       </c>
-      <c r="C9" s="174" t="n"/>
+      <c r="C9" s="192" t="n"/>
       <c r="D9" s="154" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="E9" s="175" t="n"/>
+      <c r="E9" s="193" t="n"/>
       <c r="F9" s="154" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="G9" s="175" t="n"/>
+      <c r="G9" s="193" t="n"/>
       <c r="H9" s="154" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="I9" s="175" t="n"/>
+      <c r="I9" s="193" t="n"/>
       <c r="J9" s="154" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="K9" s="175" t="n"/>
+      <c r="K9" s="193" t="n"/>
       <c r="L9" s="155" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="M9" s="176" t="n"/>
+      <c r="M9" s="194" t="n"/>
       <c r="N9" s="162" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="O9" s="157" t="n"/>
+      <c r="O9" s="195" t="n"/>
       <c r="P9" s="177" t="inlineStr">
         <is>
           <t>億</t>
@@ -1914,43 +1942,43 @@
           <t>第2四半期</t>
         </is>
       </c>
-      <c r="C10" s="178" t="n"/>
+      <c r="C10" s="196" t="n"/>
       <c r="D10" s="160" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="E10" s="178" t="n"/>
+      <c r="E10" s="196" t="n"/>
       <c r="F10" s="160" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="G10" s="178" t="n"/>
+      <c r="G10" s="196" t="n"/>
       <c r="H10" s="160" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="I10" s="178" t="n"/>
+      <c r="I10" s="196" t="n"/>
       <c r="J10" s="160" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="K10" s="178" t="n"/>
+      <c r="K10" s="196" t="n"/>
       <c r="L10" s="160" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="M10" s="179" t="n"/>
+      <c r="M10" s="197" t="n"/>
       <c r="N10" s="162" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="O10" s="163" t="n"/>
+      <c r="O10" s="198" t="n"/>
       <c r="P10" s="164" t="inlineStr">
         <is>
           <t>億</t>
@@ -1967,43 +1995,43 @@
           <t>第3四半期</t>
         </is>
       </c>
-      <c r="C11" s="178" t="n"/>
+      <c r="C11" s="196" t="n"/>
       <c r="D11" s="166" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="E11" s="178" t="n"/>
+      <c r="E11" s="196" t="n"/>
       <c r="F11" s="166" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="G11" s="178" t="n"/>
+      <c r="G11" s="196" t="n"/>
       <c r="H11" s="166" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="I11" s="178" t="n"/>
+      <c r="I11" s="196" t="n"/>
       <c r="J11" s="166" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="K11" s="178" t="n"/>
+      <c r="K11" s="196" t="n"/>
       <c r="L11" s="166" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="M11" s="179" t="n"/>
+      <c r="M11" s="197" t="n"/>
       <c r="N11" s="167" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="O11" s="163" t="n"/>
+      <c r="O11" s="198" t="n"/>
       <c r="P11" s="164" t="inlineStr">
         <is>
           <t>億</t>
@@ -2020,43 +2048,43 @@
           <t>決算</t>
         </is>
       </c>
-      <c r="C12" s="178" t="n"/>
+      <c r="C12" s="196" t="n"/>
       <c r="D12" s="163" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="E12" s="178" t="n"/>
+      <c r="E12" s="196" t="n"/>
       <c r="F12" s="163" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="G12" s="159" t="n"/>
+      <c r="G12" s="199" t="n"/>
       <c r="H12" s="163" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="I12" s="159" t="n"/>
+      <c r="I12" s="199" t="n"/>
       <c r="J12" s="163" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="K12" s="159" t="n"/>
+      <c r="K12" s="199" t="n"/>
       <c r="L12" s="163" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="M12" s="161" t="n"/>
+      <c r="M12" s="200" t="n"/>
       <c r="N12" s="167" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="O12" s="159" t="n"/>
+      <c r="O12" s="199" t="n"/>
       <c r="P12" s="164" t="inlineStr">
         <is>
           <t>億</t>
@@ -2074,37 +2102,37 @@
         </is>
       </c>
       <c r="C13" s="189">
-        <f>IFERROR(C12/C8,"")</f>
+        <f>IFERROR(TRUNC(C12/C8*1000)/1000,"")</f>
         <v/>
       </c>
       <c r="D13" s="66" t="n"/>
       <c r="E13" s="189">
-        <f>IFERROR(E12/E8,"")</f>
+        <f>IFERROR(TRUNC(E12/E8*1000)/1000,"")</f>
         <v/>
       </c>
       <c r="F13" s="66" t="n"/>
       <c r="G13" s="189">
-        <f>IFERROR(G12/G8,"")</f>
+        <f>IFERROR(TRUNC(G12/G8*1000)/1000,"")</f>
         <v/>
       </c>
       <c r="H13" s="66" t="n"/>
       <c r="I13" s="189">
-        <f>IFERROR(I12/I8,"")</f>
+        <f>IFERROR(TRUNC(I12/I8*1000)/1000,"")</f>
         <v/>
       </c>
       <c r="J13" s="66" t="n"/>
       <c r="K13" s="189">
-        <f>IFERROR(K12/K8,"")</f>
+        <f>IFERROR(TRUNC(K12/K8*1000)/1000,"")</f>
         <v/>
       </c>
       <c r="L13" s="66" t="n"/>
       <c r="M13" s="190">
-        <f>IFERROR(M12/M8,"")</f>
+        <f>IFERROR(TRUNC(M12/M8*1000)/1000,"")</f>
         <v/>
       </c>
       <c r="N13" s="22" t="n"/>
       <c r="O13" s="189">
-        <f>IFERROR(O12/O8,"")</f>
+        <f>IFERROR(TRUNC(O12/O8*1000)/1000,"")</f>
         <v/>
       </c>
       <c r="P13" s="14" t="n"/>
@@ -2514,32 +2542,32 @@
         </is>
       </c>
       <c r="C26" s="144">
-        <f>SUM(C9/C5)</f>
+        <f>TRUNC((C9/C5)*1000)/1000</f>
         <v/>
       </c>
       <c r="D26" s="145" t="n"/>
       <c r="E26" s="144">
-        <f>SUM(E9/E5)</f>
+        <f>TRUNC((E9/E5)*1000)/1000</f>
         <v/>
       </c>
       <c r="F26" s="145" t="n"/>
       <c r="G26" s="144">
-        <f>SUM(G9/G5)</f>
+        <f>TRUNC((G9/G5)*1000)/1000</f>
         <v/>
       </c>
       <c r="H26" s="145" t="n"/>
       <c r="I26" s="144">
-        <f>SUM(I9/I5)</f>
+        <f>TRUNC((I9/I5)*1000)/1000</f>
         <v/>
       </c>
       <c r="J26" s="145" t="n"/>
       <c r="K26" s="144">
-        <f>SUM(K9/K5)</f>
+        <f>TRUNC((K9/K5)*1000)/1000</f>
         <v/>
       </c>
       <c r="L26" s="145" t="n"/>
       <c r="M26" s="144">
-        <f>SUM(M9/M5)</f>
+        <f>TRUNC((M9/M5)*1000)/1000</f>
         <v/>
       </c>
       <c r="N26" s="145" t="n"/>
@@ -2555,32 +2583,32 @@
         </is>
       </c>
       <c r="C27" s="144">
-        <f>SUM(C10/C6)</f>
+        <f>TRUNC((C10/C6)*1000)/1000</f>
         <v/>
       </c>
       <c r="D27" s="146" t="n"/>
       <c r="E27" s="144">
-        <f>SUM(E10/E6)</f>
+        <f>TRUNC((E10/E6)*1000)/1000</f>
         <v/>
       </c>
       <c r="F27" s="146" t="n"/>
       <c r="G27" s="144">
-        <f>SUM(G10/G6)</f>
+        <f>TRUNC((G10/G6)*1000)/1000</f>
         <v/>
       </c>
       <c r="H27" s="146" t="n"/>
       <c r="I27" s="144">
-        <f>SUM(I10/I6)</f>
+        <f>TRUNC((I10/I6)*1000)/1000</f>
         <v/>
       </c>
       <c r="J27" s="146" t="n"/>
       <c r="K27" s="144">
-        <f>SUM(K10/K6)</f>
+        <f>TRUNC((K10/K6)*1000)/1000</f>
         <v/>
       </c>
       <c r="L27" s="146" t="n"/>
       <c r="M27" s="144">
-        <f>SUM(M10/M6)</f>
+        <f>TRUNC((M10/M6)*1000)/1000</f>
         <v/>
       </c>
       <c r="N27" s="146" t="n"/>
@@ -2596,32 +2624,32 @@
         </is>
       </c>
       <c r="C28" s="144">
-        <f>SUM(C11/C7)</f>
+        <f>TRUNC((C11/C7)*1000)/1000</f>
         <v/>
       </c>
       <c r="D28" s="147" t="n"/>
       <c r="E28" s="144">
-        <f>SUM(E11/E7)</f>
+        <f>TRUNC((E11/E7)*1000)/1000</f>
         <v/>
       </c>
       <c r="F28" s="147" t="n"/>
       <c r="G28" s="144">
-        <f>SUM(G11/G7)</f>
+        <f>TRUNC((G11/G7)*1000)/1000</f>
         <v/>
       </c>
       <c r="H28" s="147" t="n"/>
       <c r="I28" s="144">
-        <f>SUM(I11/I7)</f>
+        <f>TRUNC((I11/I7)*1000)/1000</f>
         <v/>
       </c>
       <c r="J28" s="147" t="n"/>
       <c r="K28" s="144">
-        <f>SUM(K11/K7)</f>
+        <f>TRUNC((K11/K7)*1000)/1000</f>
         <v/>
       </c>
       <c r="L28" s="147" t="n"/>
       <c r="M28" s="144">
-        <f>SUM(M11/M7)</f>
+        <f>TRUNC((M11/M7)*1000)/1000</f>
         <v/>
       </c>
       <c r="N28" s="147" t="n"/>
@@ -2637,32 +2665,32 @@
         </is>
       </c>
       <c r="C29" s="144">
-        <f>SUM(C12/C8)</f>
+        <f>TRUNC((C12/C8)*1000)/1000</f>
         <v/>
       </c>
       <c r="D29" s="148" t="n"/>
       <c r="E29" s="144">
-        <f>SUM(E12/E8)</f>
+        <f>TRUNC((E12/E8)*1000)/1000</f>
         <v/>
       </c>
       <c r="F29" s="148" t="n"/>
       <c r="G29" s="144">
-        <f>SUM(G12/G8)</f>
+        <f>TRUNC((G12/G8)*1000)/1000</f>
         <v/>
       </c>
       <c r="H29" s="148" t="n"/>
       <c r="I29" s="144">
-        <f>SUM(I12/I8)</f>
+        <f>TRUNC((I12/I8)*1000)/1000</f>
         <v/>
       </c>
       <c r="J29" s="148" t="n"/>
       <c r="K29" s="144">
-        <f>SUM(K12/K8)</f>
+        <f>TRUNC((K12/K8)*1000)/1000</f>
         <v/>
       </c>
       <c r="L29" s="148" t="n"/>
       <c r="M29" s="144">
-        <f>SUM(M12/M8)</f>
+        <f>TRUNC((M12/M8)*1000)/1000</f>
         <v/>
       </c>
       <c r="N29" s="148" t="n"/>

</xml_diff>

<commit_message>
Simplify screening UI, format market cap with commas, show ordinary profit to 1 decimal
- app.py: remove presets, saved searches, PER/ROE/dividend/margin
  filters, sector search, recently-listed filter, and the 10x-score
  card (compute_tenx_scores no longer called from the UI) per explicit
  request to simplify. Keeps the event/performance category cards,
  AND/OR toggle, and the original PBR/equity-ratio/downward-revision
  filters.
- Market cap column now shows as a comma-separated integer (e.g.
  "1,000" instead of "1000.0") via NumberColumn format="%,d".
- Execution table's ordinary-profit rows now round to 1 decimal place
  in both the written value and the template's number format (were
  inconsistently at 2 decimals in the template vs computed value).
</commit_message>
<xml_diff>
--- a/templates/execution_table_template.xlsx
+++ b/templates/execution_table_template.xlsx
@@ -15,7 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="0.00_);[Red]\(0.00\)"/>
     <numFmt numFmtId="165" formatCode="0;[Red]\(0\);\-"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -24,6 +24,7 @@
     <numFmt numFmtId="169" formatCode="0;[Red]▲0;-"/>
     <numFmt numFmtId="170" formatCode="0.0_);[Red]▲0.0_)"/>
     <numFmt numFmtId="171" formatCode="0.00;[Red]▲0.00;-"/>
+    <numFmt numFmtId="172" formatCode="0.0;[Red]▲0.0;-"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -690,7 +691,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="201">
+  <cellXfs count="210">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1256,6 +1257,33 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="171" fontId="1" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="1" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="1" fillId="0" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="1" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="1" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="1" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="1" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1885,43 +1913,43 @@
           <t>第1四半期</t>
         </is>
       </c>
-      <c r="C9" s="192" t="n"/>
+      <c r="C9" s="201" t="n"/>
       <c r="D9" s="154" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="E9" s="193" t="n"/>
+      <c r="E9" s="202" t="n"/>
       <c r="F9" s="154" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="G9" s="193" t="n"/>
+      <c r="G9" s="202" t="n"/>
       <c r="H9" s="154" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="I9" s="193" t="n"/>
+      <c r="I9" s="202" t="n"/>
       <c r="J9" s="154" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="K9" s="193" t="n"/>
+      <c r="K9" s="202" t="n"/>
       <c r="L9" s="155" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="M9" s="194" t="n"/>
+      <c r="M9" s="203" t="n"/>
       <c r="N9" s="162" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="O9" s="195" t="n"/>
+      <c r="O9" s="204" t="n"/>
       <c r="P9" s="177" t="inlineStr">
         <is>
           <t>億</t>
@@ -1942,43 +1970,43 @@
           <t>第2四半期</t>
         </is>
       </c>
-      <c r="C10" s="196" t="n"/>
+      <c r="C10" s="205" t="n"/>
       <c r="D10" s="160" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="E10" s="196" t="n"/>
+      <c r="E10" s="205" t="n"/>
       <c r="F10" s="160" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="G10" s="196" t="n"/>
+      <c r="G10" s="205" t="n"/>
       <c r="H10" s="160" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="I10" s="196" t="n"/>
+      <c r="I10" s="205" t="n"/>
       <c r="J10" s="160" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="K10" s="196" t="n"/>
+      <c r="K10" s="205" t="n"/>
       <c r="L10" s="160" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="M10" s="197" t="n"/>
+      <c r="M10" s="206" t="n"/>
       <c r="N10" s="162" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="O10" s="198" t="n"/>
+      <c r="O10" s="207" t="n"/>
       <c r="P10" s="164" t="inlineStr">
         <is>
           <t>億</t>
@@ -1995,43 +2023,43 @@
           <t>第3四半期</t>
         </is>
       </c>
-      <c r="C11" s="196" t="n"/>
+      <c r="C11" s="205" t="n"/>
       <c r="D11" s="166" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="E11" s="196" t="n"/>
+      <c r="E11" s="205" t="n"/>
       <c r="F11" s="166" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="G11" s="196" t="n"/>
+      <c r="G11" s="205" t="n"/>
       <c r="H11" s="166" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="I11" s="196" t="n"/>
+      <c r="I11" s="205" t="n"/>
       <c r="J11" s="166" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="K11" s="196" t="n"/>
+      <c r="K11" s="205" t="n"/>
       <c r="L11" s="166" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="M11" s="197" t="n"/>
+      <c r="M11" s="206" t="n"/>
       <c r="N11" s="167" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="O11" s="198" t="n"/>
+      <c r="O11" s="207" t="n"/>
       <c r="P11" s="164" t="inlineStr">
         <is>
           <t>億</t>
@@ -2048,43 +2076,43 @@
           <t>決算</t>
         </is>
       </c>
-      <c r="C12" s="196" t="n"/>
+      <c r="C12" s="205" t="n"/>
       <c r="D12" s="163" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="E12" s="196" t="n"/>
+      <c r="E12" s="205" t="n"/>
       <c r="F12" s="163" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="G12" s="199" t="n"/>
+      <c r="G12" s="208" t="n"/>
       <c r="H12" s="163" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="I12" s="199" t="n"/>
+      <c r="I12" s="208" t="n"/>
       <c r="J12" s="163" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="K12" s="199" t="n"/>
+      <c r="K12" s="208" t="n"/>
       <c r="L12" s="163" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="M12" s="200" t="n"/>
+      <c r="M12" s="209" t="n"/>
       <c r="N12" s="167" t="inlineStr">
         <is>
           <t>億</t>
         </is>
       </c>
-      <c r="O12" s="199" t="n"/>
+      <c r="O12" s="208" t="n"/>
       <c r="P12" s="164" t="inlineStr">
         <is>
           <t>億</t>

</xml_diff>

<commit_message>
Clear static explanation text from execution table remarks box
Remove the boilerplate lines under "備考:トピックス" (data-source
citations, price/forecast caveats) from the template per request,
keeping the header as an empty box for manual notes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/execution_table_template.xlsx
+++ b/templates/execution_table_template.xlsx
@@ -1723,11 +1723,7 @@
           <t>億</t>
         </is>
       </c>
-      <c r="Q5" s="158" t="inlineStr">
-        <is>
-          <t>売上・経常利益：各決算短信の累計実績（億円）</t>
-        </is>
-      </c>
+      <c r="Q5" s="158" t="n"/>
       <c r="R5" s="57" t="n"/>
       <c r="S5" s="57" t="n"/>
     </row>
@@ -1780,11 +1776,7 @@
           <t>億</t>
         </is>
       </c>
-      <c r="Q6" s="165" t="inlineStr">
-        <is>
-          <t>株価：各四半期末の終値（円、休場日は直前営業日）</t>
-        </is>
-      </c>
+      <c r="Q6" s="165" t="n"/>
       <c r="R6" s="57" t="n"/>
       <c r="S6" s="57" t="n"/>
     </row>
@@ -1837,11 +1829,7 @@
           <t>億</t>
         </is>
       </c>
-      <c r="Q7" s="164" t="inlineStr">
-        <is>
-          <t>予想年度は会社の通期予想のみ、四半期は未発表</t>
-        </is>
-      </c>
+      <c r="Q7" s="164" t="n"/>
       <c r="R7" s="57" t="n"/>
       <c r="S7" s="57" t="n"/>
     </row>
@@ -1894,11 +1882,7 @@
           <t>億</t>
         </is>
       </c>
-      <c r="Q8" s="173" t="inlineStr">
-        <is>
-          <t>業績出典：J-Quants /fins/summary</t>
-        </is>
-      </c>
+      <c r="Q8" s="173" t="n"/>
       <c r="R8" s="57" t="n"/>
       <c r="S8" s="57" t="n"/>
     </row>
@@ -1955,11 +1939,7 @@
           <t>億</t>
         </is>
       </c>
-      <c r="Q9" s="165" t="inlineStr">
-        <is>
-          <t>株価出典：J-Quants /equities/bars/daily</t>
-        </is>
-      </c>
+      <c r="Q9" s="165" t="n"/>
       <c r="R9" s="57" t="n"/>
       <c r="S9" s="57" t="n"/>
     </row>

</xml_diff>